<commit_message>
build for live production
</commit_message>
<xml_diff>
--- a/Computation/PETTYCASH LOAN.xlsx
+++ b/Computation/PETTYCASH LOAN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jeff\Desktop\peoples-information-system\Computation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F068F307-5606-45B7-B83E-2726B25B81B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEB8F5DF-910B-4A2D-9C1C-56B4AED59E78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -544,42 +544,93 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="15" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="15" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="15" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -597,57 +648,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -881,80 +881,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A1" s="71"/>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="73"/>
+      <c r="A1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="31"/>
     </row>
     <row r="2" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A2" s="34"/>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="33"/>
+      <c r="A2" s="32"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="34"/>
     </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="33"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="34"/>
     </row>
     <row r="4" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-      <c r="J4" s="33"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="34"/>
     </row>
     <row r="5" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A5" s="34"/>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="33"/>
+      <c r="A5" s="32"/>
+      <c r="B5" s="33"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="34"/>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="74" t="s">
+      <c r="A6" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="35"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="35"/>
-      <c r="I6" s="35"/>
-      <c r="J6" s="75"/>
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="39"/>
+      <c r="J6" s="40"/>
     </row>
     <row r="7" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -969,18 +969,18 @@
       <c r="J7" s="12"/>
     </row>
     <row r="8" spans="1:10" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="31"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="33"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
@@ -999,19 +999,19 @@
       <c r="B10" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="40" t="s">
+      <c r="C10" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
       <c r="F10" s="8"/>
       <c r="G10" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="H10" s="40" t="s">
+      <c r="H10" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="I10" s="41"/>
+      <c r="I10" s="42"/>
       <c r="J10" s="43"/>
     </row>
     <row r="11" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1019,21 +1019,21 @@
       <c r="B11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="69">
+      <c r="C11" s="48">
         <v>997989</v>
       </c>
-      <c r="D11" s="69"/>
-      <c r="E11" s="69"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48"/>
       <c r="F11" s="8"/>
-      <c r="G11" s="48" t="s">
+      <c r="G11" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="H11" s="31"/>
-      <c r="I11" s="67">
+      <c r="H11" s="33"/>
+      <c r="I11" s="46">
         <f>D14</f>
         <v>20000</v>
       </c>
-      <c r="J11" s="68"/>
+      <c r="J11" s="47"/>
     </row>
     <row r="12" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11"/>
@@ -1041,17 +1041,17 @@
         <v>5</v>
       </c>
       <c r="C12" s="44">
-        <v>46035</v>
-      </c>
-      <c r="D12" s="66"/>
-      <c r="E12" s="66"/>
+        <v>46042</v>
+      </c>
+      <c r="D12" s="45"/>
+      <c r="E12" s="45"/>
       <c r="F12" s="8"/>
-      <c r="G12" s="48" t="s">
+      <c r="G12" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="H12" s="31"/>
-      <c r="I12" s="70">
-        <v>46125</v>
+      <c r="H12" s="33"/>
+      <c r="I12" s="49">
+        <v>46132</v>
       </c>
       <c r="J12" s="43"/>
     </row>
@@ -1254,13 +1254,13 @@
     <row r="26" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11"/>
       <c r="B26" s="8"/>
-      <c r="C26" s="60" t="s">
+      <c r="C26" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="61"/>
-      <c r="E26" s="61"/>
-      <c r="F26" s="61"/>
-      <c r="G26" s="62"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="58"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="59"/>
       <c r="H26" s="8"/>
       <c r="I26" s="8"/>
       <c r="J26" s="12"/>
@@ -1268,11 +1268,11 @@
     <row r="27" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="11"/>
       <c r="B27" s="8"/>
-      <c r="C27" s="63"/>
-      <c r="D27" s="64"/>
-      <c r="E27" s="64"/>
-      <c r="F27" s="64"/>
-      <c r="G27" s="65"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="61"/>
+      <c r="E27" s="61"/>
+      <c r="F27" s="61"/>
+      <c r="G27" s="62"/>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
       <c r="J27" s="12"/>
@@ -1309,12 +1309,12 @@
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
       <c r="G30" s="8"/>
-      <c r="H30" s="55" t="str">
+      <c r="H30" s="50" t="str">
         <f>C10</f>
         <v>JEREMIAH N. SANDOVAL</v>
       </c>
-      <c r="I30" s="55"/>
-      <c r="J30" s="56"/>
+      <c r="I30" s="50"/>
+      <c r="J30" s="51"/>
     </row>
     <row r="31" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A31" s="11"/>
@@ -1324,11 +1324,11 @@
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
       <c r="G31" s="8"/>
-      <c r="H31" s="57" t="s">
+      <c r="H31" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="I31" s="58"/>
-      <c r="J31" s="59"/>
+      <c r="I31" s="53"/>
+      <c r="J31" s="54"/>
     </row>
     <row r="32" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A32" s="11"/>
@@ -1384,14 +1384,14 @@
         <v>42</v>
       </c>
       <c r="C36" s="8"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="30"/>
-      <c r="F36" s="30"/>
+      <c r="D36" s="55"/>
+      <c r="E36" s="56"/>
+      <c r="F36" s="56"/>
       <c r="G36" s="8"/>
-      <c r="H36" s="40" t="s">
+      <c r="H36" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="I36" s="41"/>
+      <c r="I36" s="42"/>
       <c r="J36" s="12"/>
     </row>
     <row r="37" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
@@ -1400,14 +1400,14 @@
         <v>9</v>
       </c>
       <c r="C37" s="8"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="30"/>
-      <c r="F37" s="30"/>
+      <c r="D37" s="55"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
       <c r="G37" s="8"/>
-      <c r="H37" s="29" t="s">
+      <c r="H37" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="I37" s="31"/>
+      <c r="I37" s="33"/>
       <c r="J37" s="12"/>
     </row>
     <row r="38" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
@@ -1447,44 +1447,44 @@
       <c r="J40" s="17"/>
     </row>
     <row r="41" spans="1:10" ht="13.8" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="32" t="s">
+      <c r="A41" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B41" s="31"/>
-      <c r="C41" s="31"/>
-      <c r="D41" s="31"/>
-      <c r="E41" s="31"/>
-      <c r="F41" s="31"/>
-      <c r="G41" s="31"/>
-      <c r="H41" s="31"/>
-      <c r="I41" s="31"/>
-      <c r="J41" s="33"/>
+      <c r="B41" s="33"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="33"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="33"/>
+      <c r="G41" s="33"/>
+      <c r="H41" s="33"/>
+      <c r="I41" s="33"/>
+      <c r="J41" s="34"/>
     </row>
     <row r="42" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A42" s="34"/>
-      <c r="B42" s="31"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="31"/>
-      <c r="E42" s="31"/>
-      <c r="F42" s="31"/>
-      <c r="G42" s="31"/>
-      <c r="H42" s="31"/>
-      <c r="I42" s="31"/>
-      <c r="J42" s="33"/>
+      <c r="A42" s="32"/>
+      <c r="B42" s="33"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="33"/>
+      <c r="H42" s="33"/>
+      <c r="I42" s="33"/>
+      <c r="J42" s="34"/>
     </row>
     <row r="43" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A43" s="11"/>
-      <c r="B43" s="35" t="s">
+      <c r="B43" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C43" s="31"/>
-      <c r="D43" s="31"/>
-      <c r="E43" s="31"/>
-      <c r="F43" s="31"/>
-      <c r="G43" s="31"/>
-      <c r="H43" s="31"/>
-      <c r="I43" s="31"/>
-      <c r="J43" s="33"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="33"/>
+      <c r="E43" s="33"/>
+      <c r="F43" s="33"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="33"/>
+      <c r="I43" s="33"/>
+      <c r="J43" s="34"/>
     </row>
     <row r="44" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A44" s="11"/>
@@ -1499,18 +1499,18 @@
       <c r="J44" s="12"/>
     </row>
     <row r="45" spans="1:10" ht="15" x14ac:dyDescent="0.25">
-      <c r="A45" s="39" t="s">
+      <c r="A45" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="B45" s="31"/>
-      <c r="C45" s="31"/>
-      <c r="D45" s="31"/>
-      <c r="E45" s="31"/>
-      <c r="F45" s="31"/>
-      <c r="G45" s="31"/>
-      <c r="H45" s="31"/>
-      <c r="I45" s="31"/>
-      <c r="J45" s="33"/>
+      <c r="B45" s="33"/>
+      <c r="C45" s="33"/>
+      <c r="D45" s="33"/>
+      <c r="E45" s="33"/>
+      <c r="F45" s="33"/>
+      <c r="G45" s="33"/>
+      <c r="H45" s="33"/>
+      <c r="I45" s="33"/>
+      <c r="J45" s="34"/>
     </row>
     <row r="46" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A46" s="18"/>
@@ -1529,18 +1529,18 @@
       <c r="B47" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C47" s="40" t="str">
+      <c r="C47" s="41" t="str">
         <f>C10</f>
         <v>JEREMIAH N. SANDOVAL</v>
       </c>
-      <c r="D47" s="41"/>
-      <c r="E47" s="41"/>
+      <c r="D47" s="42"/>
+      <c r="E47" s="42"/>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
       <c r="H47" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="I47" s="42"/>
+      <c r="I47" s="66"/>
       <c r="J47" s="43"/>
     </row>
     <row r="48" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
@@ -1550,15 +1550,15 @@
       </c>
       <c r="C48" s="44">
         <f>C12</f>
-        <v>46035</v>
-      </c>
-      <c r="D48" s="45"/>
-      <c r="E48" s="45"/>
+        <v>46042</v>
+      </c>
+      <c r="D48" s="67"/>
+      <c r="E48" s="67"/>
       <c r="F48" s="8"/>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
-      <c r="I48" s="46"/>
-      <c r="J48" s="47"/>
+      <c r="I48" s="68"/>
+      <c r="J48" s="69"/>
     </row>
     <row r="49" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A49" s="11"/>
@@ -1750,8 +1750,8 @@
       <c r="D61" s="3"/>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
-      <c r="G61" s="48"/>
-      <c r="H61" s="31"/>
+      <c r="G61" s="35"/>
+      <c r="H61" s="33"/>
       <c r="I61" s="8"/>
       <c r="J61" s="12"/>
     </row>
@@ -1895,13 +1895,13 @@
         <v>18</v>
       </c>
       <c r="D71" s="3"/>
-      <c r="E71" s="49" t="str">
+      <c r="E71" s="70" t="str">
         <f>C26</f>
         <v>SEVENTEEN THOUSAN PESOS</v>
       </c>
-      <c r="F71" s="50"/>
-      <c r="G71" s="50"/>
-      <c r="H71" s="51"/>
+      <c r="F71" s="71"/>
+      <c r="G71" s="71"/>
+      <c r="H71" s="72"/>
       <c r="I71" s="27">
         <f>D23</f>
         <v>17000</v>
@@ -1913,10 +1913,10 @@
       <c r="B72" s="8"/>
       <c r="C72" s="8"/>
       <c r="D72" s="21"/>
-      <c r="E72" s="52"/>
-      <c r="F72" s="53"/>
-      <c r="G72" s="53"/>
-      <c r="H72" s="54"/>
+      <c r="E72" s="73"/>
+      <c r="F72" s="74"/>
+      <c r="G72" s="74"/>
+      <c r="H72" s="75"/>
       <c r="I72" s="8"/>
       <c r="J72" s="20"/>
     </row>
@@ -1939,12 +1939,12 @@
       <c r="D74" s="8"/>
       <c r="E74" s="8"/>
       <c r="F74" s="8"/>
-      <c r="G74" s="40" t="str">
+      <c r="G74" s="41" t="str">
         <f>C10</f>
         <v>JEREMIAH N. SANDOVAL</v>
       </c>
-      <c r="H74" s="41"/>
-      <c r="I74" s="41"/>
+      <c r="H74" s="42"/>
+      <c r="I74" s="42"/>
       <c r="J74" s="12"/>
     </row>
     <row r="75" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
@@ -1954,24 +1954,24 @@
       <c r="D75" s="8"/>
       <c r="E75" s="8"/>
       <c r="F75" s="8"/>
-      <c r="G75" s="29" t="s">
+      <c r="G75" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="H75" s="31"/>
-      <c r="I75" s="31"/>
+      <c r="H75" s="33"/>
+      <c r="I75" s="33"/>
       <c r="J75" s="12"/>
     </row>
     <row r="76" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="28"/>
-      <c r="B76" s="36"/>
-      <c r="C76" s="37"/>
-      <c r="D76" s="37"/>
-      <c r="E76" s="37"/>
-      <c r="F76" s="37"/>
-      <c r="G76" s="37"/>
-      <c r="H76" s="37"/>
-      <c r="I76" s="37"/>
-      <c r="J76" s="38"/>
+      <c r="B76" s="63"/>
+      <c r="C76" s="64"/>
+      <c r="D76" s="64"/>
+      <c r="E76" s="64"/>
+      <c r="F76" s="64"/>
+      <c r="G76" s="64"/>
+      <c r="H76" s="64"/>
+      <c r="I76" s="64"/>
+      <c r="J76" s="65"/>
     </row>
     <row r="77" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3"/>
@@ -1999,24 +1999,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A1:J2"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="A4:J5"/>
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="H30:J30"/>
-    <mergeCell ref="H31:J31"/>
-    <mergeCell ref="D36:F36"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="C26:G27"/>
     <mergeCell ref="D37:F37"/>
     <mergeCell ref="H37:I37"/>
     <mergeCell ref="A41:J42"/>
@@ -2031,6 +2013,24 @@
     <mergeCell ref="G74:I74"/>
     <mergeCell ref="G75:I75"/>
     <mergeCell ref="E71:H72"/>
+    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="C26:G27"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="A1:J2"/>
+    <mergeCell ref="B3:J3"/>
+    <mergeCell ref="A4:J5"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A6:J6"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>